<commit_message>
Swiss day-first dates in the messy workbook, page 1 and page 18 (ISO dates read on their own; the mistake is now month-first); HFR labels in the workbook and template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/messy_abstraction_workbook.xlsx
+++ b/data/messy_abstraction_workbook.xlsx
@@ -383,14 +383,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TJS Outcomes Abstraction - Site A (SYNTHETIC DATA - NOT REAL PATIENTS)</t>
+          <t>HFR Ortho Outcomes Abstraction - Site A (SYNTHETIC DATA - NOT REAL PATIENTS)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Abstractor: RA | Last updated: 1/15/2026 | DO NOT SORT</t>
+          <t>Abstractor: RA | Last updated: 15.01.2026 | DO NOT SORT</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2/8/15</t>
+          <t>08.02.15</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1/25/15</t>
+          <t>25.01.15</t>
         </is>
       </c>
       <c r="M6">
@@ -648,7 +648,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5/14/15</t>
+          <t>14.05.15</t>
         </is>
       </c>
       <c r="E7">
@@ -684,7 +684,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>May 7 2015</t>
+          <t>7.5.2015</t>
         </is>
       </c>
       <c r="M7">
@@ -785,7 +785,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>August 23 2015</t>
+          <t>23.8.2015</t>
         </is>
       </c>
       <c r="E9">
@@ -855,7 +855,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>October 16 2015</t>
+          <t>16.10.2015</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>10/9/15</t>
+          <t>09.10.15</t>
         </is>
       </c>
       <c r="M11">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>8/29/16</t>
+          <t>29.08.16</t>
         </is>
       </c>
       <c r="M14">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>November 9 2016</t>
+          <t>9.11.2016</t>
         </is>
       </c>
       <c r="E17">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4/21/17</t>
+          <t>21.04.17</t>
         </is>
       </c>
       <c r="E18">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>April 22 2017</t>
+          <t>22.4.2017</t>
         </is>
       </c>
       <c r="M19">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5/17/17</t>
+          <t>17.05.17</t>
         </is>
       </c>
       <c r="E20">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>June 22 2017</t>
+          <t>22.6.2017</t>
         </is>
       </c>
       <c r="E21">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>7/30/17</t>
+          <t>30.07.17</t>
         </is>
       </c>
       <c r="M22">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2/8/19</t>
+          <t>08.02.19</t>
         </is>
       </c>
       <c r="O24">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>February 11 2018</t>
+          <t>11.2.2018</t>
         </is>
       </c>
       <c r="M25">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>February 25 2018</t>
+          <t>25.2.2018</t>
         </is>
       </c>
       <c r="M26">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>February 17 2019</t>
+          <t>17.2.2019</t>
         </is>
       </c>
       <c r="O26">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>March 12 2018</t>
+          <t>12.3.2018</t>
         </is>
       </c>
       <c r="M27">
@@ -2026,7 +2026,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>3/19/19</t>
+          <t>19.03.19</t>
         </is>
       </c>
       <c r="O27">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>4/27/19</t>
+          <t>27.04.19</t>
         </is>
       </c>
       <c r="O28">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>April 9 2018</t>
+          <t>9.4.2018</t>
         </is>
       </c>
       <c r="M29">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>6/10/18</t>
+          <t>10.06.18</t>
         </is>
       </c>
       <c r="E30">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>November 5 2018</t>
+          <t>5.11.2018</t>
         </is>
       </c>
       <c r="M31">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>January 28 2019</t>
+          <t>28.1.2019</t>
         </is>
       </c>
       <c r="M32">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2/7/19</t>
+          <t>07.02.19</t>
         </is>
       </c>
       <c r="M33">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>March 9 2019</t>
+          <t>9.3.2019</t>
         </is>
       </c>
       <c r="M34">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>April 17 2019</t>
+          <t>17.4.2019</t>
         </is>
       </c>
       <c r="E35">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>4/12/20</t>
+          <t>12.04.20</t>
         </is>
       </c>
       <c r="O35">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>May 30 2019</t>
+          <t>30.5.2019</t>
         </is>
       </c>
       <c r="E36">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>May 25 2019</t>
+          <t>25.5.2019</t>
         </is>
       </c>
       <c r="M36">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>August 13 2019</t>
+          <t>13.8.2019</t>
         </is>
       </c>
       <c r="E37">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>August 11 2019</t>
+          <t>11.8.2019</t>
         </is>
       </c>
       <c r="M38">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>September 2 2019</t>
+          <t>2.9.2019</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>8/26/19</t>
+          <t>26.08.19</t>
         </is>
       </c>
       <c r="M39">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>8/12/19</t>
+          <t>12.08.19</t>
         </is>
       </c>
       <c r="M40">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>11/18/19</t>
+          <t>18.11.19</t>
         </is>
       </c>
       <c r="M41">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>November 3 2020</t>
+          <t>3.11.2020</t>
         </is>
       </c>
       <c r="O41">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>12/19/19</t>
+          <t>19.12.19</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>January 1 2020</t>
+          <t>1.1.2020</t>
         </is>
       </c>
       <c r="E43">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>December 31 2020</t>
+          <t>31.12.2020</t>
         </is>
       </c>
       <c r="O43">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>1/12/20</t>
+          <t>12.01.20</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3265,7 +3265,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>1/18/20</t>
+          <t>18.01.20</t>
         </is>
       </c>
       <c r="M45">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>1/12/21</t>
+          <t>12.01.21</t>
         </is>
       </c>
       <c r="O45">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2/4/20</t>
+          <t>04.02.20</t>
         </is>
       </c>
       <c r="M46">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>2/6/21</t>
+          <t>06.02.21</t>
         </is>
       </c>
       <c r="O46">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>3/21/20</t>
+          <t>21.03.20</t>
         </is>
       </c>
       <c r="E47">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>3/18/20</t>
+          <t>18.03.20</t>
         </is>
       </c>
       <c r="M48">
@@ -3484,7 +3484,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>4/10/21</t>
+          <t>10.04.21</t>
         </is>
       </c>
       <c r="O48">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>April 21 2020</t>
+          <t>21.4.2020</t>
         </is>
       </c>
       <c r="E49">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>May 10 2021</t>
+          <t>10.5.2021</t>
         </is>
       </c>
       <c r="O49">
@@ -3611,7 +3611,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>April 11 2020</t>
+          <t>11.4.2020</t>
         </is>
       </c>
       <c r="M50">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>May 6 2021</t>
+          <t>6.5.2021</t>
         </is>
       </c>
       <c r="O50">
@@ -3685,7 +3685,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>5/26/21</t>
+          <t>26.05.21</t>
         </is>
       </c>
       <c r="O51">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>June 24 2020</t>
+          <t>24.6.2020</t>
         </is>
       </c>
       <c r="E52">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>September 18 2020</t>
+          <t>18.9.2020</t>
         </is>
       </c>
       <c r="M53">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>10/22/20</t>
+          <t>22.10.20</t>
         </is>
       </c>
       <c r="E54">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="N55" t="inlineStr">
         <is>
-          <t>December 14 2021</t>
+          <t>14.12.2021</t>
         </is>
       </c>
       <c r="O55">
@@ -3982,7 +3982,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>January 24 2021</t>
+          <t>24.1.2021</t>
         </is>
       </c>
       <c r="E56">
@@ -4091,7 +4091,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>3/5/22</t>
+          <t>05.03.22</t>
         </is>
       </c>
       <c r="O57">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>October 25 2021</t>
+          <t>25.10.2021</t>
         </is>
       </c>
       <c r="M59">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>February 25 2018</t>
+          <t>25.2.2018</t>
         </is>
       </c>
       <c r="M60">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>February 17 2019</t>
+          <t>17.2.2019</t>
         </is>
       </c>
       <c r="O60">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>1/27/23</t>
+          <t>27.01.23</t>
         </is>
       </c>
       <c r="O61">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>1/27/23</t>
+          <t>27.01.23</t>
         </is>
       </c>
       <c r="O62">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>March 3 2022</t>
+          <t>3.3.2022</t>
         </is>
       </c>
       <c r="E63">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>2/23/22</t>
+          <t>23.02.22</t>
         </is>
       </c>
       <c r="M63">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>8/29/22</t>
+          <t>29.08.22</t>
         </is>
       </c>
       <c r="E64">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>August 26 2022</t>
+          <t>26.8.2022</t>
         </is>
       </c>
       <c r="M64">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>11/15/23</t>
+          <t>15.11.23</t>
         </is>
       </c>
       <c r="O65">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>6/8/23</t>
+          <t>08.06.23</t>
         </is>
       </c>
       <c r="E66">
@@ -4781,14 +4781,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>TJS Outcomes Abstraction - Site B (SYNTHETIC DATA - NOT REAL PATIENTS)</t>
+          <t>HFR Ortho Outcomes Abstraction - Site B (SYNTHETIC DATA - NOT REAL PATIENTS)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Abstractor: RA | Last updated: 1/15/2026 | DO NOT SORT</t>
+          <t>Abstractor: RA | Last updated: 15.01.2026 | DO NOT SORT</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>June 10 2015</t>
+          <t>10.6.2015</t>
         </is>
       </c>
       <c r="N5">
@@ -4966,7 +4966,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>June 23 2016</t>
+          <t>23.6.2016</t>
         </is>
       </c>
       <c r="P5">
@@ -5171,7 +5171,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>November 1 2015</t>
+          <t>1.11.2015</t>
         </is>
       </c>
       <c r="N8">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>December 16 2016</t>
+          <t>16.12.2016</t>
         </is>
       </c>
       <c r="P9">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>January 27 2017</t>
+          <t>27.1.2017</t>
         </is>
       </c>
       <c r="P10">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>February 4 2016</t>
+          <t>4.2.2016</t>
         </is>
       </c>
       <c r="E11">
@@ -5465,7 +5465,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2/6/17</t>
+          <t>06.02.17</t>
         </is>
       </c>
       <c r="P12">
@@ -5495,7 +5495,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3/29/16</t>
+          <t>29.03.16</t>
         </is>
       </c>
       <c r="E13">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4/11/16</t>
+          <t>11.04.16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>May 8 2017</t>
+          <t>8.5.2017</t>
         </is>
       </c>
       <c r="P14">
@@ -5676,7 +5676,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>5/25/16</t>
+          <t>25.05.16</t>
         </is>
       </c>
       <c r="N15">
@@ -5757,7 +5757,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>6/12/17</t>
+          <t>12.06.17</t>
         </is>
       </c>
       <c r="P16">
@@ -5820,7 +5820,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>6/17/17</t>
+          <t>17.06.17</t>
         </is>
       </c>
       <c r="P17">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>7/16/16</t>
+          <t>16.07.16</t>
         </is>
       </c>
       <c r="N18">
@@ -5958,7 +5958,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>10/16/17</t>
+          <t>16.10.17</t>
         </is>
       </c>
       <c r="P19">
@@ -6017,7 +6017,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>September 23 2016</t>
+          <t>23.9.2016</t>
         </is>
       </c>
       <c r="N20">
@@ -6055,7 +6055,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>October 27 2016</t>
+          <t>27.10.2016</t>
         </is>
       </c>
       <c r="E21">
@@ -6096,7 +6096,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>10/1/16</t>
+          <t>01.10.16</t>
         </is>
       </c>
       <c r="N21">
@@ -6127,7 +6127,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>11/12/16</t>
+          <t>12.11.16</t>
         </is>
       </c>
       <c r="E22">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>11/7/16</t>
+          <t>07.11.16</t>
         </is>
       </c>
       <c r="N22">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2/14/17</t>
+          <t>14.02.17</t>
         </is>
       </c>
       <c r="E24">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>February 14 2018</t>
+          <t>14.2.2018</t>
         </is>
       </c>
       <c r="P24">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>5/31/18</t>
+          <t>31.05.18</t>
         </is>
       </c>
       <c r="P25">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>September 22 2017</t>
+          <t>22.9.2017</t>
         </is>
       </c>
       <c r="E28">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>9/11/18</t>
+          <t>11.09.18</t>
         </is>
       </c>
       <c r="P28">
@@ -6661,7 +6661,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>October 29 2018</t>
+          <t>29.10.2018</t>
         </is>
       </c>
       <c r="P29">
@@ -6730,7 +6730,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>11/21/17</t>
+          <t>21.11.17</t>
         </is>
       </c>
       <c r="N30">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2/18/19</t>
+          <t>18.02.19</t>
         </is>
       </c>
       <c r="N32">
@@ -7045,7 +7045,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>October 28 2019</t>
+          <t>28.10.2019</t>
         </is>
       </c>
       <c r="E35">
@@ -7160,7 +7160,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>10/29/19</t>
+          <t>29.10.19</t>
         </is>
       </c>
       <c r="N36">
@@ -7193,7 +7193,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>December 14 2019</t>
+          <t>14.12.2019</t>
         </is>
       </c>
       <c r="E37">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>12/11/19</t>
+          <t>11.12.19</t>
         </is>
       </c>
       <c r="N37">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>12/5/19</t>
+          <t>05.12.19</t>
         </is>
       </c>
       <c r="N38">
@@ -7344,7 +7344,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2/11/20</t>
+          <t>11.02.20</t>
         </is>
       </c>
       <c r="E39">
@@ -7411,7 +7411,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>4/13/20</t>
+          <t>13.04.20</t>
         </is>
       </c>
       <c r="E40">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>3/19/21</t>
+          <t>19.03.21</t>
         </is>
       </c>
       <c r="P40">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>September 16 2020</t>
+          <t>16.9.2020</t>
         </is>
       </c>
       <c r="E41">
@@ -7525,7 +7525,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>October 15 2021</t>
+          <t>15.10.2021</t>
         </is>
       </c>
       <c r="P41">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>10/22/20</t>
+          <t>22.10.20</t>
         </is>
       </c>
       <c r="E42">
@@ -7595,7 +7595,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>10/22/21</t>
+          <t>22.10.21</t>
         </is>
       </c>
       <c r="P42">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>November 20 2020</t>
+          <t>20.11.2020</t>
         </is>
       </c>
       <c r="E43">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2/25/21</t>
+          <t>25.02.21</t>
         </is>
       </c>
       <c r="E44">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>3/29/21</t>
+          <t>29.03.21</t>
         </is>
       </c>
       <c r="E45">
@@ -7804,7 +7804,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>March 29 2022</t>
+          <t>29.3.2022</t>
         </is>
       </c>
       <c r="P45">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>April 6 2021</t>
+          <t>6.4.2021</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>April 2 2021</t>
+          <t>2.4.2021</t>
         </is>
       </c>
       <c r="N46">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>April 28 2022</t>
+          <t>28.4.2022</t>
         </is>
       </c>
       <c r="P46">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>5/14/21</t>
+          <t>14.05.21</t>
         </is>
       </c>
       <c r="E47">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>May 3 2021</t>
+          <t>3.5.2021</t>
         </is>
       </c>
       <c r="N47">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>June 20 2021</t>
+          <t>20.6.2021</t>
         </is>
       </c>
       <c r="E48">
@@ -8015,7 +8015,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>6/7/21</t>
+          <t>07.06.21</t>
         </is>
       </c>
       <c r="N48">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>5/22/22</t>
+          <t>22.05.22</t>
         </is>
       </c>
       <c r="P48">
@@ -8233,7 +8233,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>October 19 2021</t>
+          <t>19.10.2021</t>
         </is>
       </c>
       <c r="N51">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2/11/22</t>
+          <t>11.02.22</t>
         </is>
       </c>
       <c r="E52">
@@ -8306,7 +8306,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>2/10/22</t>
+          <t>10.02.22</t>
         </is>
       </c>
       <c r="N52">
@@ -8458,7 +8458,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>7/21/23</t>
+          <t>21.07.23</t>
         </is>
       </c>
       <c r="P54">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>10/15/22</t>
+          <t>15.10.22</t>
         </is>
       </c>
       <c r="N56">
@@ -8820,7 +8820,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>4/11/16</t>
+          <t>11.04.16</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>May 8 2017</t>
+          <t>8.5.2017</t>
         </is>
       </c>
       <c r="P60">
@@ -8890,7 +8890,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>November 20 2020</t>
+          <t>20.11.2020</t>
         </is>
       </c>
       <c r="E61">
@@ -8996,7 +8996,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>April 7 2024</t>
+          <t>7.4.2024</t>
         </is>
       </c>
       <c r="P62">
@@ -9127,7 +9127,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>10/9/23</t>
+          <t>09.10.23</t>
         </is>
       </c>
       <c r="N64">
@@ -9135,7 +9135,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>November 1 2024</t>
+          <t>1.11.2024</t>
         </is>
       </c>
       <c r="P64">
@@ -9160,7 +9160,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>July 8 2024</t>
+          <t>8.7.2024</t>
         </is>
       </c>
       <c r="E65">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>July 6 2024</t>
+          <t>6.7.2024</t>
         </is>
       </c>
       <c r="N65">

</xml_diff>